<commit_message>
feat: modelo vial — ciclovia+base granular, calzada rigida+excav, 20 keywords nuevos
- ciclovia genera base_granular_e200mm e=150mm (faltaba en formula original)
  → interseccion demo mejora de -3.5% a -1.2% vs referencial $200 MM
- calzada_rigida genera excavacion_tierra_comun (losa+sub_base depth)
- Nueva seccion 'ciclovia' en _DEFAULT_SECCIONES y secciones_civiles.yaml
- Nuevos keywords calzada_granular: ESPALDON, BERMA GRANULAR, CAMINO LATERAL
- Nuevos keywords colector: TUBERIA HDPE, TUBERIA CORRUGADA, SUBCOLECTOR
- Nuevos keywords muro (entrada temprana): ENROCADO, ENROCAMIENTO, MURO GAVION
- Nuevos keywords ciclovia: CICLOPISTA, VIA CICLISTA, SENDA CICLISTA
- Nuevo keyword calzada_rigida: CALZADA HORMIGON, HORMIGON CALZADA
- Orden _VIAL_CATS: calzada_rigida y enrocado/escollera antes de reglas generales
- 150 tests pasando (+16 nuevos tests)

https://claude.ai/code/session_016BR4zVrkucAbqsHCWRUVRh
</commit_message>
<xml_diff>
--- a/interseccion_cubicacion.xlsx
+++ b/interseccion_cubicacion.xlsx
@@ -527,7 +527,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-18 03:03</t>
+          <t>2026-05-18 03:12</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>$ 129.700.000</t>
+          <t>$ 132.780.000</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>$ 32.425.000</t>
+          <t>$ 33.195.000</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>$ 162.125.000</t>
+          <t>$ 165.975.000</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>$ 30.803.750</t>
+          <t>$ 31.535.250</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>$ 192.928.750 CLP</t>
+          <t>$ 197.510.250 CLP</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>$ 41.171 CLP/m²</t>
+          <t>$ 42.149 CLP/m²</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3504</v>
+        <v>4064</v>
       </c>
       <c r="E5" t="n">
         <v>5500</v>

</xml_diff>